<commit_message>
Add CuspAI and Wonderful (manual finds, verified mega-rounds) to master and near-miss register
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TE8a9ptd2NGPUtY6iZfzkb
</commit_message>
<xml_diff>
--- a/reports/F1-Near-Misses-Added-2026-09.xlsx
+++ b/reports/F1-Near-Misses-Added-2026-09.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="NEAR MISSES ALL CATEGORIES" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NEAR MISSES ALL CATEGORIES" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -92,7 +92,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -108,6 +108,12 @@
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -475,7 +481,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P251"/>
+  <dimension ref="A1:P253"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -663,7 +669,6 @@
           <t>Large capital backing from a major insurance holding group to scale a specialty P&amp;C underwriting platform, one of the few nine-figure insurtech capital events in a quiet quarter for the sector.</t>
         </is>
       </c>
-      <c r="P6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
@@ -742,7 +747,6 @@
           <t>Riding the AI-data-center power boom with a fresh $550M for factory expansion, Antora is scaling from engineering story to industrial brand -- global sponsorship visibility supports enterprise sales into heavy-industry and hyperscaler accounts.</t>
         </is>
       </c>
-      <c r="P8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="5" t="n">
@@ -814,7 +818,6 @@
           <t>A domestic solar manufacturer scaling capacity fourfold on fresh nine-figure capital is building an American-manufacturing brand story -- sponsorship visibility supports both policy narrative and B2B customer trust as it competes with Asian incumbents.</t>
         </is>
       </c>
-      <c r="P9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="5" t="n">
@@ -886,7 +889,6 @@
           <t>A $13B home-battery unicorn expanding beyond Texas needs consumer-facing brand equity fast -- global sports sponsorship is a proven playbook for battery/EV-adjacent brands moving from early adopters to mass market.</t>
         </is>
       </c>
-      <c r="P10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="5" t="n">
@@ -958,7 +960,6 @@
           <t>A newly minted multi-billion-dollar nuclear brand needs to build public confidence in advanced reactor technology beyond its data-center customer base -- a global, safety-and-performance-obsessed platform like F1 supports that trust narrative.</t>
         </is>
       </c>
-      <c r="P11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="5" t="n">
@@ -1030,7 +1031,6 @@
           <t>Newly public, well-capitalized geothermal leader riding AI-driven power demand; needs consumer/brand visibility beyond utility-scale B2B deals, fitting F1's clean-energy and grid-innovation storylines.</t>
         </is>
       </c>
-      <c r="P12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="5" t="n">
@@ -1102,7 +1102,6 @@
           <t>Flagship European green-steel/industrial-decarbonization story with massive capital deployment, aligning with F1's sustainability and advanced-manufacturing narrative.</t>
         </is>
       </c>
-      <c r="P13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="7" t="n">
@@ -1326,7 +1325,6 @@
           <t>A near-unicorn-scale capital injection for 'power at the speed of American innovation' signals an aggressive brand-building phase for a young energy-infrastructure company that needs credibility with industrial and hyperscaler customers.</t>
         </is>
       </c>
-      <c r="P16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="5" t="n">
@@ -1398,7 +1396,6 @@
           <t>Marquee, Twilio-founder-led fusion bet with huge capital and a bold engineering narrative well suited to F1's cutting-edge-technology sponsorship positioning.</t>
         </is>
       </c>
-      <c r="P17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="5" t="n">
@@ -1470,7 +1467,6 @@
           <t>Newly capitalized grid-storage platform tackling the AI power crunch; early-stage brand with room to attach to a high-visibility sustainability/tech platform like F1.</t>
         </is>
       </c>
-      <c r="P18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="5" t="n">
@@ -1542,7 +1538,6 @@
           <t>A software-first critical-minerals unicorn supplying the EV/AI/defense supply chain is building a modern brand identity distinct from traditional mining -- global sponsorship visibility supports both capital raising and offtake partner recruitment.</t>
         </is>
       </c>
-      <c r="P19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="7" t="n">
@@ -1697,7 +1692,6 @@
           <t>High-profile fashion brand exiting LVMH for an independent, growth-focused ownership structure with capital earmarked to rebuild global visibility.</t>
         </is>
       </c>
-      <c r="P22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="5" t="n">
@@ -1769,7 +1763,6 @@
           <t>Marquee luxury fragrance/beauty business moving to a growth-focused global operator; luxury fragrance houses are increasingly active in high-end motorsport sponsorship.</t>
         </is>
       </c>
-      <c r="P23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="4" t="inlineStr">
@@ -1848,7 +1841,6 @@
           <t>Iconic F&amp;B brand freshly capitalized under a growth-focused new parent, fitting the profile of brands seeking mainstream visibility platforms.</t>
         </is>
       </c>
-      <c r="P25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="5" t="n">
@@ -1920,7 +1912,6 @@
           <t>Fast-growing D2C-turned-national sauce brand acquired with clear growth mandate; capital-flush F&amp;B brands are prime new-sponsor prospects.</t>
         </is>
       </c>
-      <c r="P26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="5" t="n">
@@ -1992,7 +1983,6 @@
           <t>Fresh strategic ownership with an explicit mandate to scale a premium D2C food brand nationally; matches profile of growth-capitalized consumer brands entering sponsorship conversations.</t>
         </is>
       </c>
-      <c r="P27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="4" t="inlineStr">
@@ -2063,7 +2053,6 @@
           <t>A strategic domestic HPC brand seeking China-market prestige; the Shanghai GP offers a high-visibility local platform for building consumer and enterprise trust.</t>
         </is>
       </c>
-      <c r="P29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="4" t="inlineStr">
@@ -2134,7 +2123,6 @@
           <t>~$14.7B revenue, ~75k employees; agency holding companies use marquee sports sponsorships to showcase integrated brand-building capability to clients, mirroring rival Publicis's existing F1 tie.</t>
         </is>
       </c>
-      <c r="P31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="5" t="n">
@@ -2198,7 +2186,6 @@
           <t>~$1.4B FY2024 revenue; Yelp is expanding ad services for auto-services and hospitality SMBs, sectors that cluster around F1 race weekends, and has no existing sports sponsorship to anchor brand campaigns.</t>
         </is>
       </c>
-      <c r="P32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="5" t="n">
@@ -2262,7 +2249,6 @@
           <t>World's largest ad holding company (~$15B revenue, ~100k staff); its agencies already run automotive/tech accounts and F1's global, affluent, brand-safe audience fits WPP's cross-agency pitch to CMOs.</t>
         </is>
       </c>
-      <c r="P33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="5" t="n">
@@ -2326,7 +2312,6 @@
           <t>~$10.7B revenue, ~55k staff; IPG (merging with Omnicom) needs high-visibility platforms to prove data-driven media capability, and F1's premium global reach fits its client roster of autos/finance brands.</t>
         </is>
       </c>
-      <c r="P34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="5" t="n">
@@ -2390,7 +2375,6 @@
           <t>~$9B revenue, ~66k employees; Dentsu is the exclusive sales agent for Japanese GP commercial rights and has deep motorsport ties, making direct sponsorship a natural extension of its F1 relationship.</t>
         </is>
       </c>
-      <c r="P35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="4" t="inlineStr">
@@ -2469,7 +2453,6 @@
           <t>UK fixed-income/credit data analytics platform newly crossing $1B valuation, part of a wave of UK fintech unicorns with fresh capital for global expansion.</t>
         </is>
       </c>
-      <c r="P37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="5" t="n">
@@ -2541,7 +2524,6 @@
           <t>Massive early-stage raise for an enterprise AI/data platform founded by a high-profile ex-xAI co-founder, a headline-grabbing brand story.</t>
         </is>
       </c>
-      <c r="P38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="5" t="n">
@@ -2613,7 +2595,6 @@
           <t>Record-setting YC unicorn with a compelling growth story, appealing for a splashy early sponsorship before it scales further.</t>
         </is>
       </c>
-      <c r="P39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" s="5" t="n">
@@ -2685,7 +2666,6 @@
           <t>AI code-review platform used by 17,000 customers newly reaching unicorn status, well-positioned to invest in brand awareness.</t>
         </is>
       </c>
-      <c r="P40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" s="5" t="n">
@@ -2757,7 +2737,6 @@
           <t>Extremely fast-growing AI coding unicorn seeking to build a global enterprise developer brand rapidly.</t>
         </is>
       </c>
-      <c r="P41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" s="5" t="n">
@@ -2829,7 +2808,6 @@
           <t>Freshly unicorn-status enterprise AI infrastructure startup backed by Nvidia/Intel/Dell Capital, in brand-building mode.</t>
         </is>
       </c>
-      <c r="P42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" s="4" t="inlineStr">
@@ -2908,7 +2886,6 @@
           <t>Indonesia's top consumer fintech brand going public, giving it fresh capital and a mandate for regional brand-building right as F1 courts Southeast Asian audiences and sponsors.</t>
         </is>
       </c>
-      <c r="P44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" s="5" t="n">
@@ -2980,7 +2957,6 @@
           <t>Singapore's cross-border payments infrastructure champion being absorbed into a major global fintech (Circle), creating a newly resourced combined brand relevant to F1's Singapore GP market.</t>
         </is>
       </c>
-      <c r="P45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" s="5" t="n">
@@ -3052,7 +3028,6 @@
           <t>Global card-issuing infrastructure provider raising a large round earmarked for product development, talent and global expansion, positioning it for a bigger international brand push.</t>
         </is>
       </c>
-      <c r="P46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" s="5" t="n">
@@ -3124,7 +3099,6 @@
           <t>UK digital business bank hitting unicorn status with fresh capital, fitting F1's UK/European banking sponsor category and growth-stage marketing budgets.</t>
         </is>
       </c>
-      <c r="P47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" s="5" t="n">
@@ -3196,7 +3170,6 @@
           <t>Digital wealth manager reaching unicorn status on a $150M round led by a top growth-equity firm, targeting the HNW client base that overlaps with F1's fan demographics.</t>
         </is>
       </c>
-      <c r="P48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" s="5" t="n">
@@ -3268,7 +3241,6 @@
           <t>Newly-crowned Indian lending unicorn raising a large round explicitly to prep for an IPO, indicating a scaling marketing and brand budget in a market F1 is actively growing.</t>
         </is>
       </c>
-      <c r="P49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" s="5" t="n">
@@ -3340,7 +3312,6 @@
           <t>One of Mexico's largest-ever fintech rounds and a genuine LatAm champion with a mass-market consumer brand; well suited to a Mexico GP-anchored regional partnership.</t>
         </is>
       </c>
-      <c r="P50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" s="5" t="n">
@@ -3412,7 +3383,6 @@
           <t>Doubled its valuation to $2B on a mega Series E, giving the workplace-savings infrastructure platform fresh growth capital and brand-building ambitions.</t>
         </is>
       </c>
-      <c r="P51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" s="5" t="n">
@@ -3484,7 +3454,6 @@
           <t>Target of the third-biggest US bank M&amp;A deal since 2010; large regional bank undergoing a major capital-markets event, distinct from the acquiring sponsor-excluded entity.</t>
         </is>
       </c>
-      <c r="P52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" s="5" t="n">
@@ -3556,7 +3525,6 @@
           <t>Freshly capitalized UAE fintech champion in a fast-growing Gulf digital-banking niche; strong candidate for a Gulf-region F1 partnership tied to the Abu Dhabi Grand Prix, distinct from existing airline/logistics Gulf sponsors.</t>
         </is>
       </c>
-      <c r="P53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" s="5" t="n">
@@ -3628,7 +3596,6 @@
           <t>San Francisco business-banking platform crossing $1B valuation and reaching unicorn status, a fast-growing fintech with new marquee-investor capital to deploy on brand growth.</t>
         </is>
       </c>
-      <c r="P54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" s="4" t="inlineStr">
@@ -3699,7 +3666,6 @@
           <t>An Italian tech champion with Monza/Imola home-market ties; its EU data-sovereignty message fits Europe-first team sponsorship narratives.</t>
         </is>
       </c>
-      <c r="P56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" s="5" t="n">
@@ -3763,7 +3729,6 @@
           <t>An ultra-low-latency storage pitch parallels F1's real-time data demands; its compact size mirrors smaller technical partners already in the paddock (e.g., JetCool, Motivair).</t>
         </is>
       </c>
-      <c r="P57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" s="4" t="inlineStr">
@@ -3842,7 +3807,6 @@
           <t>Indonesia's leading online stock/investment trading platform, newly capitalized and expanding into stablecoin rails — Southeast Asia is a priority growth region for F1 (Singapore GP).</t>
         </is>
       </c>
-      <c r="P59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" s="5" t="n">
@@ -3914,7 +3878,6 @@
           <t>Large, long-established UK SME lender expanding funding capacity, indicating a bigger marketing budget for brand-building sponsorships.</t>
         </is>
       </c>
-      <c r="P60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" s="5" t="n">
@@ -3986,7 +3949,6 @@
           <t>Well-capitalized wealthtech platform connecting financial advisors to alternative investments, serving the high-net-worth advisor audience F1 hospitality targets.</t>
         </is>
       </c>
-      <c r="P61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" s="5" t="n">
@@ -4058,7 +4020,6 @@
           <t>One of the largest single insurtech raises of 2026, giving the company a large marketing war chest as it scales nationally.</t>
         </is>
       </c>
-      <c r="P62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" s="5" t="n">
@@ -4130,7 +4091,6 @@
           <t>Fast-scaling co-branded credit card issuing platform with a huge new balance sheet, reflecting strong institutional confidence and growth ambition.</t>
         </is>
       </c>
-      <c r="P63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" s="5" t="n">
@@ -4202,7 +4162,6 @@
           <t>UK-based insurtech premium-finance platform with a large new capital base and pan-European ambitions.</t>
         </is>
       </c>
-      <c r="P64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" s="5" t="n">
@@ -4274,7 +4233,6 @@
           <t>Institutional FX/crypto exchange with $8.2T in trading volume expanding into stablecoin collateral and cross-asset trading with fresh capital, giving it budget and a growth narrative for global brand marketing.</t>
         </is>
       </c>
-      <c r="P65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" s="7" t="n">
@@ -4422,7 +4380,6 @@
           <t>Stablecoin-powered neobank that just crossed the $1B mark, Dubai-based in a region with deep F1 ties (Abu Dhabi GP) and strong crypto-sponsorship appetite.</t>
         </is>
       </c>
-      <c r="P67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" s="5" t="n">
@@ -4494,7 +4451,6 @@
           <t>Global cross-border payments giant raising ahead of an eventual IPO, headquartered in Singapore (an existing F1 race market) with ambitions to expand merchant/consumer payment brand across Asia and the Middle East.</t>
         </is>
       </c>
-      <c r="P68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" s="5" t="n">
@@ -4566,7 +4522,6 @@
           <t>Global wealth-management technology platform with $2.5T on platform, backed by major long-term institutional investors and fresh capital for its turnaround/growth plan.</t>
         </is>
       </c>
-      <c r="P69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" s="5" t="n">
@@ -4638,7 +4593,6 @@
           <t>Global payment terminal/acquiring leader based in France with fresh capital, long tied to major retail and card-network partnerships.</t>
         </is>
       </c>
-      <c r="P70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" s="5" t="n">
@@ -4710,7 +4664,6 @@
           <t>Miami-based, WhatsApp-first remittance unicorn serving Latino immigrants across the Americas — a demographic and geography (Miami GP, LatAm fan growth) highly relevant to F1's US expansion.</t>
         </is>
       </c>
-      <c r="P71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" s="5" t="n">
@@ -4782,7 +4735,6 @@
           <t>Consumer-facing payments/rewards brand with fresh capital and a hospitality/lifestyle angle that could pair well with F1's paddock club and fan-experience sponsorships.</t>
         </is>
       </c>
-      <c r="P72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" s="5" t="n">
@@ -4854,7 +4806,6 @@
           <t>Corporate card and spend-management fintech with fresh growth capital, a segment (Ramp, Brex, Moss) increasingly active in sports sponsorship.</t>
         </is>
       </c>
-      <c r="P73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" s="5" t="n">
@@ -4926,7 +4877,6 @@
           <t>Instant money-movement infrastructure provider for banks and fintechs, raising capital while pursuing a bank charter — a growth-stage payments brand building national visibility.</t>
         </is>
       </c>
-      <c r="P74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" s="7" t="n">
@@ -5074,7 +5024,6 @@
           <t>Stablecoin card/payments infrastructure unicorn with 38x card-volume growth and 200+ bank/fintech partners; global consumer-facing crypto payments brand seeking mainstream visibility.</t>
         </is>
       </c>
-      <c r="P76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" s="4" t="inlineStr">
@@ -5153,7 +5102,6 @@
           <t>Well-funded foundational AI lab building brand presence early, before wider market awareness catches up.</t>
         </is>
       </c>
-      <c r="P78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" s="5" t="n">
@@ -5225,7 +5173,6 @@
           <t>Enormous seed round for a stealth foundational AI lab signals deep pockets and future brand-building needs.</t>
         </is>
       </c>
-      <c r="P79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" s="5" t="n">
@@ -5297,7 +5244,6 @@
           <t>Fresh unicorn in AI-safety/interpretability needing enterprise credibility; sponsorship could position it alongside trust/safety-minded engineering brands on the grid.</t>
         </is>
       </c>
-      <c r="P80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" s="5" t="n">
@@ -5369,7 +5315,6 @@
           <t>Flush, high-profile new entrant explicitly positioning around teamwork/communication tech - resonant with F1's pit-wall/team-communication storyline and needs a splashy brand launch.</t>
         </is>
       </c>
-      <c r="P81" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" s="5" t="n">
@@ -5441,7 +5386,6 @@
           <t>UK-based, newly launched with record capital and needs brand visibility fast; David Silver's RL pedigree (AlphaGo) gives a natural "learning from experience" storyline for a UK-rooted F1 team.</t>
         </is>
       </c>
-      <c r="P82" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" s="4" t="inlineStr">
@@ -5520,7 +5464,6 @@
           <t>Endpoint-security vendor on an unbroken multi-year growth streak, using large late-stage capital to fund premium global brand campaigns.</t>
         </is>
       </c>
-      <c r="P84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" s="5" t="n">
@@ -5592,7 +5535,6 @@
           <t>Fresh corporate rebrand (ActiveFence to Alice) paired with a large raise, a classic moment for a brand to seek high-visibility sponsorship.</t>
         </is>
       </c>
-      <c r="P85" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" s="5" t="n">
@@ -5664,7 +5606,6 @@
           <t>Newly crossed unicorn in SaaS security for AI agents, a fast-growing category needing enterprise brand credibility.</t>
         </is>
       </c>
-      <c r="P86" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" s="5" t="n">
@@ -5736,7 +5677,6 @@
           <t>Offensive cyber-operations vendor with a large 2026 raise, entering a high-visibility growth and branding phase.</t>
         </is>
       </c>
-      <c r="P87" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" s="5" t="n">
@@ -5808,7 +5748,6 @@
           <t>Breakout endpoint-security startup with an outsized Series A, positioned for an aggressive brand-awareness push.</t>
         </is>
       </c>
-      <c r="P88" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" s="5" t="n">
@@ -5880,7 +5819,6 @@
           <t>Threat-intelligence vendor with one of the largest cyber funding rounds of the year, scaling enterprise go-to-market and brand reach.</t>
         </is>
       </c>
-      <c r="P89" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" s="5" t="n">
@@ -5952,7 +5890,6 @@
           <t>Consumer privacy brand pushing into enterprise with sports-sponsorship appetite already shown (NFLPA investor/partner); a natural comp for testing F1 fan-facing sponsorship.</t>
         </is>
       </c>
-      <c r="P90" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" s="5" t="n">
@@ -6024,7 +5961,6 @@
           <t>Brand-new unicorn in AI-native cyber defense; needs fast market credibility and F1's global enterprise-buyer audience is a strong fit for a young cybersecurity challenger.</t>
         </is>
       </c>
-      <c r="P91" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" s="4" t="inlineStr">
@@ -6103,7 +6039,6 @@
           <t>Splunk &amp; Dynatrace on grid — rival pressure</t>
         </is>
       </c>
-      <c r="P93" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" s="4" t="inlineStr">
@@ -6174,7 +6109,6 @@
           <t>BME-listed European hotel group (~EUR2B revenue) with strong presence near several European F1 venues (Spain, Italy); a logical race-market hospitality partner.</t>
         </is>
       </c>
-      <c r="P95" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" s="5" t="n">
@@ -6238,7 +6172,6 @@
           <t>SET-listed hospitality group (~$2B+ revenue) spanning luxury (Anantara) to midscale (NH Hotels) brands across Asia-Pacific and Europe, both regions with F1 race calendars.</t>
         </is>
       </c>
-      <c r="P96" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" s="5" t="n">
@@ -6302,7 +6235,6 @@
           <t>US hotel operator (~$3B revenue) formed via the Extended Stay America merger; scale clears the core revenue gate and it lacks any current motorsport sponsorship.</t>
         </is>
       </c>
-      <c r="P97" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" s="5" t="n">
@@ -6366,7 +6298,6 @@
           <t>French all-inclusive resort brand under Fosun Tourism Group, with ~65 resorts worldwide and staffing well above the core employee gate; premium leisure positioning fits F1's lifestyle hospitality tier.</t>
         </is>
       </c>
-      <c r="P98" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" s="4" t="inlineStr">
@@ -6445,7 +6376,6 @@
           <t>A SoftBank/OpenAI-backed power-infrastructure platform heading toward a public listing without operating data-center capacity yet needs a strong, trust-building brand story for public investors -- global sponsorship is a fast route to that visibility.</t>
         </is>
       </c>
-      <c r="P100" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" s="5" t="n">
@@ -6517,7 +6447,6 @@
           <t>Mature AI networking infrastructure vendor scaling internationally, well-suited to a global marketing platform.</t>
         </is>
       </c>
-      <c r="P101" t="inlineStr"/>
     </row>
     <row r="102">
       <c r="A102" s="5" t="n">
@@ -6589,7 +6518,6 @@
           <t>India's newest, best-capitalized AI infrastructure champion; strong fit for F1's India growth push and a compelling 'built for scale' brand story around the Indian Grand Prix return.</t>
         </is>
       </c>
-      <c r="P102" t="inlineStr"/>
     </row>
     <row r="103">
       <c r="A103" s="5" t="n">
@@ -6661,7 +6589,6 @@
           <t>Newly-flush AI networking infrastructure firm scaling to meet data center demand, open to brand-building spend.</t>
         </is>
       </c>
-      <c r="P103" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" s="5" t="n">
@@ -6733,7 +6660,6 @@
           <t>Massive stealth-exit round for an AI infrastructure company gives it a big budget for early brand positioning.</t>
         </is>
       </c>
-      <c r="P104" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" s="7" t="n">
@@ -6881,7 +6807,6 @@
           <t>Newly unicorn AI cloud infrastructure company with a fresh war chest for market entry and brand building.</t>
         </is>
       </c>
-      <c r="P106" t="inlineStr"/>
     </row>
     <row r="107">
       <c r="A107" s="5" t="n">
@@ -6953,7 +6878,6 @@
           <t>Founded by the creators of vLLM, the dominant open-source inference engine; needs brand-building beyond the devtools community as it commercializes.</t>
         </is>
       </c>
-      <c r="P107" t="inlineStr"/>
     </row>
     <row r="108">
       <c r="A108" s="5" t="n">
@@ -7025,7 +6949,6 @@
           <t>Networking-infrastructure unicorn built around power efficiency and reliability at scale - directly analogous to F1's own high-reliability, low-latency data network needs.</t>
         </is>
       </c>
-      <c r="P108" t="inlineStr"/>
     </row>
     <row r="109">
       <c r="A109" s="7" t="n">
@@ -7173,7 +7096,6 @@
           <t>New unicorn selling global, low-latency AI compute; positioning around reliability and speed at scale echoes F1's real-time performance-engineering story.</t>
         </is>
       </c>
-      <c r="P110" t="inlineStr"/>
     </row>
     <row r="111">
       <c r="A111" s="5" t="n">
@@ -7245,7 +7167,6 @@
           <t>Fast-rising space/AI-infrastructure unicorn (17 months from YC demo day) with a bold narrative and fresh capital for brand-building.</t>
         </is>
       </c>
-      <c r="P111" t="inlineStr"/>
     </row>
     <row r="112">
       <c r="A112" s="4" t="inlineStr">
@@ -7400,7 +7321,6 @@
           <t>One of India's largest B2B marketplaces recapitalizing ahead of an IPO, a high-visibility turnaround story that could use F1's brand-building platform as it repositions for public markets.</t>
         </is>
       </c>
-      <c r="P114" t="inlineStr"/>
     </row>
     <row r="115">
       <c r="A115" s="5" t="n">
@@ -7472,7 +7392,6 @@
           <t>Newly minted $20B marketplace with huge fresh marketing budget and a Gen-Z/collector audience overlapping F1's fastest-growing fan demographic; live-commerce format pairs naturally with race-day merchandise drops.</t>
         </is>
       </c>
-      <c r="P115" t="inlineStr"/>
     </row>
     <row r="116">
       <c r="A116" s="5" t="n">
@@ -7544,7 +7463,6 @@
           <t>Premium agtech brand (vertical-farmed strawberries) with a luxury, sustainability-forward positioning that fits F1's paddock hospitality and sustainability sponsorship inventory; agtech is an open category among F1 partners.</t>
         </is>
       </c>
-      <c r="P116" t="inlineStr"/>
     </row>
     <row r="117">
       <c r="A117" s="5" t="n">
@@ -7616,7 +7534,6 @@
           <t>Large consumer-products consolidation creating a bigger, better-capitalized bedding/home group with brand-visibility incentives.</t>
         </is>
       </c>
-      <c r="P117" t="inlineStr"/>
     </row>
     <row r="118">
       <c r="A118" s="4" t="inlineStr">
@@ -7687,7 +7604,6 @@
           <t>World's oldest sovereign wealth fund (~$800B+ AUM) with no current F1 presence; fits the special sovereign-entity allowance and represents a Gulf state not yet visible on the grid via its investment arm.</t>
         </is>
       </c>
-      <c r="P119" t="inlineStr"/>
     </row>
     <row r="120">
       <c r="A120" s="5" t="n">
@@ -7751,7 +7667,6 @@
           <t>Saudi Arabia's ~$925B sovereign wealth fund and owner/backer of NEOM, Qiddiya, ROSHN, Riyadh Air and SURJ Sports Investment; sovereign backing alone clears the core gate and it is not itself a current F1 sponsor.</t>
         </is>
       </c>
-      <c r="P120" t="inlineStr"/>
     </row>
     <row r="121">
       <c r="A121" s="5" t="n">
@@ -7815,7 +7730,6 @@
           <t>Qatar's sovereign wealth fund (~$500B AUM); state-linked capital pool distinct from Qatar Airways/stc which are already excluded as current sponsors, giving Qatar a second sovereign-vehicle entry point into F1.</t>
         </is>
       </c>
-      <c r="P121" t="inlineStr"/>
     </row>
     <row r="122">
       <c r="A122" s="5" t="n">
@@ -7879,7 +7793,6 @@
           <t>One of the world's largest sovereign wealth funds (est. $900B+ AUM); Abu Dhabi already hosts a race weekend, and ADIA is a distinct entity from Mubadala (excluded), offering an untapped state-capital sponsor angle.</t>
         </is>
       </c>
-      <c r="P122" t="inlineStr"/>
     </row>
     <row r="123">
       <c r="A123" s="5" t="n">
@@ -7943,7 +7856,6 @@
           <t>Dubai's principal sovereign investment arm holding stakes across Emirates, Emirates NBD and DEWA; distinct legal entity from Emirates (excluded) and not currently an F1 sponsor itself.</t>
         </is>
       </c>
-      <c r="P123" t="inlineStr"/>
     </row>
     <row r="124">
       <c r="A124" s="5" t="n">
@@ -8007,7 +7919,6 @@
           <t>New PIF-owned Saudi national carrier launching commercial flights in 2025/26; sovereign-backed with a global brand-building mandate, and separate from Saudia/Qatar Airways-type exclusions.</t>
         </is>
       </c>
-      <c r="P124" t="inlineStr"/>
     </row>
     <row r="125">
       <c r="A125" s="5" t="n">
@@ -8071,7 +7982,6 @@
           <t>Saudi entertainment/events group behind Riyadh Season, WWE Arabia and other giga-events tied to the state's Vision 2030 sports push; publicly reported revenue not disclosed, so flagged as sentiment pending confirmed financials rather than assumed core.</t>
         </is>
       </c>
-      <c r="P125" t="inlineStr"/>
     </row>
     <row r="126">
       <c r="A126" s="4" t="inlineStr">
@@ -8142,7 +8052,6 @@
           <t>Global leader in advanced high-strength and fossil-free ('HYBRIT') steel used in vehicle safety structures, matching F1's own sustainability and lightweight-safety engineering narrative.</t>
         </is>
       </c>
-      <c r="P127" t="inlineStr"/>
     </row>
     <row r="128">
       <c r="A128" s="5" t="n">
@@ -8206,7 +8115,6 @@
           <t>World's largest steelmaker by output outside China, with major automotive-steel supply business and global brand recognition suited to F1's international sponsor tier.</t>
         </is>
       </c>
-      <c r="P128" t="inlineStr"/>
     </row>
     <row r="129">
       <c r="A129" s="4" t="inlineStr">
@@ -8285,7 +8193,6 @@
           <t>Newly public Indian logistics champion with a strong debut and fresh public-market capital, exactly the kind of high-visibility regional IPO F1 targets as it builds its India fan base and sponsor pipeline.</t>
         </is>
       </c>
-      <c r="P130" t="inlineStr"/>
     </row>
     <row r="131">
       <c r="A131" s="5" t="n">
@@ -8357,7 +8264,6 @@
           <t>New logistics unicorn in the flexible-warehousing space; distinct niche from DHL's F1 partnership (marketplace/network model vs. carrier), giving F1 a non-conflicting logistics-tech prospect with fresh unicorn press cycle.</t>
         </is>
       </c>
-      <c r="P131" t="inlineStr"/>
     </row>
     <row r="132">
       <c r="A132" s="5" t="n">
@@ -8429,7 +8335,6 @@
           <t>Agentic AI platform with 150+ enterprise customers and fresh capital eyeing broader brand awareness.</t>
         </is>
       </c>
-      <c r="P132" t="inlineStr"/>
     </row>
     <row r="133">
       <c r="A133" s="4" t="inlineStr">
@@ -8508,7 +8413,6 @@
           <t>Rapidly scaling AI biotech with pharma partnerships and fresh capital looking to build global brand credibility.</t>
         </is>
       </c>
-      <c r="P134" t="inlineStr"/>
     </row>
     <row r="135">
       <c r="A135" s="5" t="n">
@@ -8580,7 +8484,6 @@
           <t>Generative video/creative AI platform with global consumer reach fits a high-visibility motorsport sponsorship.</t>
         </is>
       </c>
-      <c r="P135" t="inlineStr"/>
     </row>
     <row r="136">
       <c r="A136" s="5" t="n">
@@ -8652,7 +8555,6 @@
           <t>Viral consumer AI assistant with a young, global fanbase is a strong fit for F1's younger, tech-savvy audience.</t>
         </is>
       </c>
-      <c r="P136" t="inlineStr"/>
     </row>
     <row r="137">
       <c r="A137" s="5" t="n">
@@ -8724,7 +8626,6 @@
           <t>Category-leading generative 3D platform with global creator base wants marquee brand visibility for consumer growth.</t>
         </is>
       </c>
-      <c r="P137" t="inlineStr"/>
     </row>
     <row r="138">
       <c r="A138" s="5" t="n">
@@ -8796,7 +8697,6 @@
           <t>Well-funded AI tools platform for small businesses expanding its customer base and brand reach.</t>
         </is>
       </c>
-      <c r="P138" t="inlineStr"/>
     </row>
     <row r="139">
       <c r="A139" s="5" t="n">
@@ -8868,7 +8768,6 @@
           <t>Consumer-facing AI voice app with athlete investors already on the cap table, primed for lifestyle/sports brand plays.</t>
         </is>
       </c>
-      <c r="P139" t="inlineStr"/>
     </row>
     <row r="140">
       <c r="A140" s="5" t="n">
@@ -8940,7 +8839,6 @@
           <t>Newly-minted unicorn in agentic enterprise finance software looking to build brand trust with large customers.</t>
         </is>
       </c>
-      <c r="P140" t="inlineStr"/>
     </row>
     <row r="141">
       <c r="A141" s="4" t="inlineStr">
@@ -9019,7 +8917,6 @@
           <t>GDS Holdings' Southeast Asia data-center brand landing a multi-billion-dollar raise for regional hyperscale expansion — an operating infrastructure brand (not a pure real-estate SPV) with global growth ambitions.</t>
         </is>
       </c>
-      <c r="P142" t="inlineStr"/>
     </row>
     <row r="143">
       <c r="A143" s="5" t="n">
@@ -9091,7 +8988,6 @@
           <t>APAC-based AI infrastructure operator flush with Nvidia/Blackstone-backed mega-capital, pivoting from bitcoin mining to a global 'AI factory' brand story that needs visibility as it expands into new APAC markets, including Australia — natural home-market tie-in to the Australian GP.</t>
         </is>
       </c>
-      <c r="P143" t="inlineStr"/>
     </row>
     <row r="144">
       <c r="A144" s="5" t="n">
@@ -9163,7 +9059,6 @@
           <t>Founded by noted chip architect Jim Keller and freshly valued at $3.7B, Fab2 is trying to reinvent domestic chip manufacturing -- a high-profile global platform fits its ambition to become a household name in reshored advanced manufacturing.</t>
         </is>
       </c>
-      <c r="P144" t="inlineStr"/>
     </row>
     <row r="145">
       <c r="A145" s="5" t="n">
@@ -9235,7 +9130,6 @@
           <t>Well-capitalized agentic-AI infrastructure player seeking marquee visibility to win enterprise inference contracts.</t>
         </is>
       </c>
-      <c r="P145" t="inlineStr"/>
     </row>
     <row r="146">
       <c r="A146" s="5" t="n">
@@ -9307,7 +9201,6 @@
           <t>Spanish satellite-to-phone connectivity operator raising a step-change round — a consumer-facing 'connect anywhere' story from a Spanish GP host country, well suited to global broadcast sponsorship.</t>
         </is>
       </c>
-      <c r="P146" t="inlineStr"/>
     </row>
     <row r="147">
       <c r="A147" s="5" t="n">
@@ -9379,7 +9272,6 @@
           <t>Newly-unicorn AI compute silicon startup seeking brand differentiation in a crowded chip market.</t>
         </is>
       </c>
-      <c r="P147" t="inlineStr"/>
     </row>
     <row r="148">
       <c r="A148" s="5" t="n">
@@ -9451,7 +9343,6 @@
           <t>British in-memory-compute chip challenger with an explosive valuation run and a marquee AI-lab customer — a breakout UK tech story looking for global brand elevation, well suited to the British GP.</t>
         </is>
       </c>
-      <c r="P148" t="inlineStr"/>
     </row>
     <row r="149">
       <c r="A149" s="5" t="n">
@@ -9523,7 +9414,6 @@
           <t>Two-year-old London photonic-AI-chip startup tripling its valuation with UK sovereign backing — a rapidly emerging British deep-tech brand well matched to the British GP home audience.</t>
         </is>
       </c>
-      <c r="P149" t="inlineStr"/>
     </row>
     <row r="150">
       <c r="A150" s="5" t="n">
@@ -9595,7 +9485,6 @@
           <t>AI-for-chip-design pitch (AlphaChip founders) maps directly to F1's engineering-performance narrative and semiconductor/engineering sponsorship slot.</t>
         </is>
       </c>
-      <c r="P150" t="inlineStr"/>
     </row>
     <row r="151">
       <c r="A151" s="4" t="inlineStr">
@@ -9674,7 +9563,6 @@
           <t>Singapore-based AI video/entertainment unicorn with fresh nine-figure capital and ambitions in interactive content, fitting both the SEA-champion and media/gaming search criteria for F1 sponsorship prospecting.</t>
         </is>
       </c>
-      <c r="P152" t="inlineStr"/>
     </row>
     <row r="153">
       <c r="A153" s="5" t="n">
@@ -9746,7 +9634,6 @@
           <t>Well-funded generative 3D/gaming content platform positioned to supply game studios and virtual-experience builders, a fit for F1's gaming and esports partner ecosystem.</t>
         </is>
       </c>
-      <c r="P153" t="inlineStr"/>
     </row>
     <row r="154">
       <c r="A154" s="4" t="inlineStr">
@@ -9817,7 +9704,6 @@
           <t>Publicly traded (NYSE: PLOW) market leader in snow/ice control attachments; revenue clears the $200M threshold and its 'performance in extreme conditions' brand story parallels F1 engineering marketing.</t>
         </is>
       </c>
-      <c r="P155" t="inlineStr"/>
     </row>
     <row r="156">
       <c r="A156" s="5" t="n">
@@ -9881,7 +9767,6 @@
           <t>Largest independent U.S. transit-bus builder (reported ~30-40% U.S. market share, acquired by American Industrial Partners in 2021); no public financials, but scale of output implies multi-hundred-million-dollar revenue, and its electrification push mirrors F1's sustainability narrative.</t>
         </is>
       </c>
-      <c r="P156" t="inlineStr"/>
     </row>
     <row r="157">
       <c r="A157" s="5" t="n">
@@ -9945,7 +9830,6 @@
           <t>World's largest forklift/material-handling manufacturer with deep precision-engineering credentials and Toyota Group manufacturing prestige, giving a natural entry point despite Toyota Motor itself sitting outside F1.</t>
         </is>
       </c>
-      <c r="P157" t="inlineStr"/>
     </row>
     <row r="158">
       <c r="A158" s="4" t="inlineStr">
@@ -10024,7 +9908,6 @@
           <t>Well-capitalized AI risk-intelligence firm expanding into new verticals, seeking broader brand recognition.</t>
         </is>
       </c>
-      <c r="P159" t="inlineStr"/>
     </row>
     <row r="160">
       <c r="A160" s="4" t="inlineStr">
@@ -10179,7 +10062,6 @@
           <t>Freshly public defense-sensing company (formed from the Accelint/Vitesse Systems merger) with a near-$1B backlog, entering the post-IPO phase where sponsorship brand plays are common.</t>
         </is>
       </c>
-      <c r="P162" t="inlineStr"/>
     </row>
     <row r="163">
       <c r="A163" s="7" t="n">
@@ -10327,7 +10209,6 @@
           <t>Newly minted counter-drone unicorn needing to build brand recognition beyond DoD buyers.</t>
         </is>
       </c>
-      <c r="P164" t="inlineStr"/>
     </row>
     <row r="165">
       <c r="A165" s="7" t="n">
@@ -10475,7 +10356,6 @@
           <t>Backed by marquee tech investors and opening a new manufacturing facility; a scaling space company positioned to invest in brand-building.</t>
         </is>
       </c>
-      <c r="P166" t="inlineStr"/>
     </row>
     <row r="167">
       <c r="A167" s="4" t="inlineStr">
@@ -10546,7 +10426,6 @@
           <t>Raised well over $150M cumulative venture funding for AI robotics; a growth-stage AI narrative that fits F1's data-driven performance story.</t>
         </is>
       </c>
-      <c r="P168" t="inlineStr"/>
     </row>
     <row r="169">
       <c r="A169" s="4" t="inlineStr">
@@ -10617,7 +10496,6 @@
           <t>China remains a priority growth market for F1; a leading domestic edge/CDN provider offers activation reach independent of the Western hyperscalers already engaged.</t>
         </is>
       </c>
-      <c r="P170" t="inlineStr"/>
     </row>
     <row r="171">
       <c r="A171" s="4" t="inlineStr">
@@ -10696,7 +10574,6 @@
           <t>Newly-crossed unicorn proptech brand with fresh capital for national expansion and consumer awareness building, a classic profile for first-time motorsport sponsorship to build trust and scale.</t>
         </is>
       </c>
-      <c r="P172" t="inlineStr"/>
     </row>
     <row r="173">
       <c r="A173" s="5" t="n">
@@ -10768,7 +10645,6 @@
           <t>India's newest proptech unicorn with a large sales and brand-marketing footprint; proptech is an open F1 sponsorship category and India remains a priority growth market for the sport.</t>
         </is>
       </c>
-      <c r="P173" t="inlineStr"/>
     </row>
     <row r="174">
       <c r="A174" s="4" t="inlineStr">
@@ -10847,7 +10723,6 @@
           <t>Newly public sustainable-fashion brand with fresh IPO capital and a global growth mandate; F1's younger, affluent, increasingly female-skewing fanbase (esp. via Drive to Survive) is a strong demographic match for Reformation's core customer.</t>
         </is>
       </c>
-      <c r="P175" t="inlineStr"/>
     </row>
     <row r="176">
       <c r="A176" s="5" t="n">
@@ -10919,7 +10794,6 @@
           <t>Canada's largest wine producer, newly backed by a deep-pocketed financial holding company, fits the wine/spirits hospitality lane that F1 has cultivated (paddock club, race-weekend activations) and needs a growth story post-buyout.</t>
         </is>
       </c>
-      <c r="P176" t="inlineStr"/>
     </row>
     <row r="177">
       <c r="A177" s="5" t="n">
@@ -10991,7 +10865,6 @@
           <t>L'Oreal-backed, fast-growing Indian D2C beauty platform gains global ambitions right as F1 deepens its presence in India/Asia — a strategic regional sponsorship growth story.</t>
         </is>
       </c>
-      <c r="P177" t="inlineStr"/>
     </row>
     <row r="178">
       <c r="A178" s="5" t="n">
@@ -11063,7 +10936,6 @@
           <t>Newly Danone-backed performance-nutrition brand with an Asia-Pacific growth mandate lines up with F1's expansion in that region and the sport's growing roster of protein/performance-nutrition partners.</t>
         </is>
       </c>
-      <c r="P178" t="inlineStr"/>
     </row>
     <row r="179">
       <c r="A179" s="5" t="n">
@@ -11135,7 +11007,6 @@
           <t>A newly carved-out, PE-backed portfolio of household wellness/supplement brands will need a standalone growth and brand-building strategy — prime timing for a motorsport sponsorship pitch.</t>
         </is>
       </c>
-      <c r="P179" t="inlineStr"/>
     </row>
     <row r="180">
       <c r="A180" s="5" t="n">
@@ -11207,7 +11078,6 @@
           <t>Iconic premium-water brands (Perrier, S.Pellegrino) newly under a growth-oriented PE structure looking for global relaunch momentum — a strong hospitality/paddock-club fit for F1's luxury beverage lane.</t>
         </is>
       </c>
-      <c r="P180" t="inlineStr"/>
     </row>
     <row r="181">
       <c r="A181" s="5" t="n">
@@ -11279,7 +11149,6 @@
           <t>Newly PE-backed premium skincare brand with fresh growth capital and a physician-endorsed, science-led positioning that fits F1's expanding luxury/lifestyle sponsor roster.</t>
         </is>
       </c>
-      <c r="P181" t="inlineStr"/>
     </row>
     <row r="182">
       <c r="A182" s="5" t="n">
@@ -11351,7 +11220,6 @@
           <t>A stable of iconic UK household food brands changing hands to Europe's largest dairy group signals fresh investment appetite for consumer-brand visibility around F1's British Grand Prix market.</t>
         </is>
       </c>
-      <c r="P182" t="inlineStr"/>
     </row>
     <row r="183">
       <c r="A183" s="5" t="n">
@@ -11423,7 +11291,6 @@
           <t>A well-known D2C menswear brand now backed by a century-old apparel platform with retail scale-up resources fits F1's smart-casual, lifestyle-apparel sponsorship lane.</t>
         </is>
       </c>
-      <c r="P183" t="inlineStr"/>
     </row>
     <row r="184">
       <c r="A184" s="7" t="n">
@@ -11571,7 +11438,6 @@
           <t>Marc Lore's fast-growing national food platform is aggressively brand-building city by city with a huge new raise; a global, high-visibility platform like F1 fits its ambition to become a household consumer name.</t>
         </is>
       </c>
-      <c r="P185" t="inlineStr"/>
     </row>
     <row r="186">
       <c r="A186" s="5" t="n">
@@ -11643,7 +11509,6 @@
           <t>Fast-scaling national psychiatry/mental-health brand with fresh growth capital and consumer-facing ambitions; fits F1's push into health &amp; wellness sponsors seeking mainstream brand visibility.</t>
         </is>
       </c>
-      <c r="P186" t="inlineStr"/>
     </row>
     <row r="187">
       <c r="A187" s="5" t="n">
@@ -11715,7 +11580,6 @@
           <t>Large capital infusion into a data/performance-health platform aligns with F1's telemetry-and-performance storytelling and sponsor-activation opportunities.</t>
         </is>
       </c>
-      <c r="P187" t="inlineStr"/>
     </row>
     <row r="188">
       <c r="A188" s="5" t="n">
@@ -11787,7 +11651,6 @@
           <t>One of the world's largest fast-fashion retailers just went public and needs to rehabilitate/build global brand image — a high-visibility platform like F1 offers exactly the kind of mainstream credibility a newly listed Shein would want.</t>
         </is>
       </c>
-      <c r="P188" t="inlineStr"/>
     </row>
     <row r="189">
       <c r="A189" s="5" t="n">
@@ -11859,7 +11722,6 @@
           <t>Already co-founded by a global sports icon (David Beckham) and sitting on a $1B facility earmarked specifically for marketing spend, IM8 is arguably the single best-primed prospect on this list for a major motorsport sponsorship activation.</t>
         </is>
       </c>
-      <c r="P189" t="inlineStr"/>
     </row>
     <row r="190">
       <c r="A190" s="5" t="n">
@@ -11931,7 +11793,6 @@
           <t>A social-media-native, youth-skewing spirits brand newly backed by a major US drinks group with global scaling ambitions mirrors the kind of fast-growth alcohol brand F1 has courted for hospitality tie-ins.</t>
         </is>
       </c>
-      <c r="P190" t="inlineStr"/>
     </row>
     <row r="191">
       <c r="A191" s="5" t="n">
@@ -12003,7 +11864,6 @@
           <t>An athletic-performance-associated OTC brand (long used by athletes for airflow) freshly acquired for over $1B by a growth-focused OTC consolidator — a strong logical tie-in to motorsport performance/endurance messaging.</t>
         </is>
       </c>
-      <c r="P191" t="inlineStr"/>
     </row>
     <row r="192">
       <c r="A192" s="5" t="n">
@@ -12075,7 +11935,6 @@
           <t>A celebrity-founded, design-forward travel brand now backed by the world's largest luggage company is exactly the kind of fresh-capital travel-lifestyle brand that fits F1's jet-set, globe-trotting audience.</t>
         </is>
       </c>
-      <c r="P192" t="inlineStr"/>
     </row>
     <row r="193">
       <c r="A193" s="5" t="n">
@@ -12147,7 +12006,6 @@
           <t>A premium hydration/functional-beverage brand freshly scaled by a public strategic acquirer fits F1's hydration/electrolyte sponsor lane and its push into Southeast Asian markets.</t>
         </is>
       </c>
-      <c r="P193" t="inlineStr"/>
     </row>
     <row r="194">
       <c r="A194" s="7" t="n">
@@ -12371,7 +12229,6 @@
           <t>GLP-1/weight-management telehealth is one of the hottest-funded health verticals; fresh $200M and a &gt;$2B valuation signal budget for a marquee consumer-marketing platform like F1.</t>
         </is>
       </c>
-      <c r="P196" t="inlineStr"/>
     </row>
     <row r="197">
       <c r="A197" s="5" t="n">
@@ -12443,7 +12300,6 @@
           <t>Newly-minted unicorn in the fast-growing women's health category; capital and unicorn status support a national brand-awareness push that F1's broad demographic reach could serve.</t>
         </is>
       </c>
-      <c r="P197" t="inlineStr"/>
     </row>
     <row r="198">
       <c r="A198" s="5" t="n">
@@ -12515,7 +12371,6 @@
           <t>Newly crossed $1B+ valuation in the booming GLP-1/nutrition space; growth-stage consumer health brand with capital to spend on brand-building platforms.</t>
         </is>
       </c>
-      <c r="P198" t="inlineStr"/>
     </row>
     <row r="199">
       <c r="A199" s="5" t="n">
@@ -12587,7 +12442,6 @@
           <t>Large fresh PE injection into a leading fitness/wellness consumer platform; fits F1's growing lifestyle/wellness sponsorship inventory and gives access to an affluent, active fan demographic.</t>
         </is>
       </c>
-      <c r="P199" t="inlineStr"/>
     </row>
     <row r="200">
       <c r="A200" s="5" t="n">
@@ -12659,7 +12513,6 @@
           <t>Enormous Series A for AI-driven wellness gives it outsized capital to build consumer brand trust quickly.</t>
         </is>
       </c>
-      <c r="P200" t="inlineStr"/>
     </row>
     <row r="201">
       <c r="A201" s="5" t="n">
@@ -12731,7 +12584,6 @@
           <t>Fast-scaling, cash-flush CPG portfolio (David, HallPass) with a performance/discipline brand ethos and celebrity-founder (Peter Rahal, RXBAR) profile that fits F1's fitness-adjacent, aspirational audience and has fresh capital earmarked for national growth marketing.</t>
         </is>
       </c>
-      <c r="P201" t="inlineStr"/>
     </row>
     <row r="202">
       <c r="A202" s="5" t="n">
@@ -12803,7 +12655,6 @@
           <t>Backed by high-profile tech figures (Brian Armstrong, Blake Byers) and riding the longevity wave that F1-adjacent brands (Oura, Whoop) have already monetized via motorsport; large war chest signals it will need consumer-facing brand building as it commercializes.</t>
         </is>
       </c>
-      <c r="P202" t="inlineStr"/>
     </row>
     <row r="203">
       <c r="A203" s="4" t="inlineStr">
@@ -12874,7 +12725,6 @@
           <t>World's largest automaker by volume; currently absent from F1 (competes in WEC/WRC instead), leaving a rare open lane for a top-tier OEM sponsorship or technical-partner conversation.</t>
         </is>
       </c>
-      <c r="P204" t="inlineStr"/>
     </row>
     <row r="205">
       <c r="A205" s="5" t="n">
@@ -12938,7 +12788,6 @@
           <t>Fast-growing global OEM investing heavily in performance/EV sub-brands and international sports sponsorship (already active in football, e.g. FIFA), with no existing F1 commitment.</t>
         </is>
       </c>
-      <c r="P205" t="inlineStr"/>
     </row>
     <row r="206">
       <c r="A206" s="5" t="n">
@@ -13002,7 +12851,6 @@
           <t>Largest U.S. new/used vehicle retailer by revenue, scaling internationally (UK acquisitions); consumer-facing auto retail brands fit F1's growing U.S. fan base and Grand Prix expansion.</t>
         </is>
       </c>
-      <c r="P206" t="inlineStr"/>
     </row>
     <row r="207">
       <c r="A207" s="5" t="n">
@@ -13066,7 +12914,6 @@
           <t>One of the largest U.S. automotive retailers, with a consumer marketing budget well suited to reach F1's fast-growing American audience post Netflix 'Drive to Survive'.</t>
         </is>
       </c>
-      <c r="P207" t="inlineStr"/>
     </row>
     <row r="208">
       <c r="A208" s="5" t="n">
@@ -13130,7 +12977,6 @@
           <t>Global dealership group under the Penske brand, whose motorsport-steeped ownership (Team Penske in IndyCar/NASCAR) gives an existing racing-marketing culture that could extend into F1 sponsorship.</t>
         </is>
       </c>
-      <c r="P208" t="inlineStr"/>
     </row>
     <row r="209">
       <c r="A209" s="5" t="n">
@@ -13194,7 +13040,6 @@
           <t>Large publicly traded U.S. dealer group actively expanding via acquisition, fitting the profile of consumer-automotive brands using F1's U.S. growth to reach car buyers.</t>
         </is>
       </c>
-      <c r="P209" t="inlineStr"/>
     </row>
     <row r="210">
       <c r="A210" s="4" t="inlineStr">
@@ -13265,7 +13110,6 @@
           <t>~$12B revenue industrial gas and hardgoods distributor with a large-scale industrial customer base fitting an F1 supply-chain sponsorship.</t>
         </is>
       </c>
-      <c r="P211" t="inlineStr"/>
     </row>
     <row r="212">
       <c r="A212" s="4" t="inlineStr">
@@ -13336,7 +13180,6 @@
           <t>~$400M FY2024 revenue; serves insurers and asset managers, a client base already well represented among F1 sponsors, giving Clearwater a plausible entry point to reach the same institutional-investor decision-makers.</t>
         </is>
       </c>
-      <c r="P213" t="inlineStr"/>
     </row>
     <row r="214">
       <c r="A214" s="4" t="inlineStr">
@@ -13415,7 +13258,6 @@
           <t>European launch startup with strong industrial backing and a Spain HQ, offering a natural regional tie-in for F1's Spanish/European fanbase and engineering story.</t>
         </is>
       </c>
-      <c r="P215" t="inlineStr"/>
     </row>
     <row r="216">
       <c r="A216" s="4" t="inlineStr">
@@ -13486,7 +13328,6 @@
           <t>Family-owned premium appliance maker (~EUR5.4B revenue, 23k+ staff) with a 'Immer Besser' precision-engineering positioning that fits well alongside other premium-lifestyle F1 partners.</t>
         </is>
       </c>
-      <c r="P217" t="inlineStr"/>
     </row>
     <row r="218">
       <c r="A218" s="5" t="n">
@@ -13550,7 +13391,6 @@
           <t>BIST-listed appliance maker (~EUR6B revenue) with pan-European distribution and prior sports-sponsorship experience (football); global media reach of F1 suits its brand-building ambitions in new markets.</t>
         </is>
       </c>
-      <c r="P218" t="inlineStr"/>
     </row>
     <row r="219">
       <c r="A219" s="4" t="inlineStr">
@@ -13629,7 +13469,6 @@
           <t>Brazil's newest AI-native unicorn and a rare LatAm vertical-AI success story, positioned for a regional partnership around F1's Sao Paulo Grand Prix.</t>
         </is>
       </c>
-      <c r="P220" t="inlineStr"/>
     </row>
     <row r="221">
       <c r="A221" s="4" t="inlineStr">
@@ -13700,7 +13539,6 @@
           <t>SK Group specialty-gas arm supplying global chipmakers; Korea regional champion niche-gas play overlooked on the current list.</t>
         </is>
       </c>
-      <c r="P222" t="inlineStr"/>
     </row>
     <row r="223">
       <c r="A223" s="5" t="n">
@@ -13764,7 +13602,6 @@
           <t>Major Korean welding-consumables/equipment maker (shielding-gas welding); fabrication/engineering-partner fit for F1 chassis manufacturing sponsorship.</t>
         </is>
       </c>
-      <c r="P223" t="inlineStr"/>
     </row>
     <row r="224">
       <c r="A224" s="5" t="n">
@@ -13828,7 +13665,6 @@
           <t>Longtime top-tier LNG liquefaction technology/EPC provider; hydrogen-carrier (MCH) technology pioneer aligning with F1 sustainable-fuel messaging.</t>
         </is>
       </c>
-      <c r="P224" t="inlineStr"/>
     </row>
     <row r="225">
       <c r="A225" s="5" t="n">
@@ -13892,7 +13728,6 @@
           <t>Builds LNG/hydrogen and industrial-gas processing plants globally; engineering-scale brand suited to F1's energy-transition sponsorship angle.</t>
         </is>
       </c>
-      <c r="P225" t="inlineStr"/>
     </row>
     <row r="226">
       <c r="A226" s="5" t="n">
@@ -13956,7 +13791,6 @@
           <t>Australian engineering major active in gas processing, hydrogen and carbon-capture projects; regional-champion catch (APAC/Oceania) for the category.</t>
         </is>
       </c>
-      <c r="P226" t="inlineStr"/>
     </row>
     <row r="227">
       <c r="A227" s="4" t="inlineStr">
@@ -14035,7 +13869,6 @@
           <t>Newly public national furniture retailer with fresh capital markets access and investor pressure to build brand awareness at scale.</t>
         </is>
       </c>
-      <c r="P228" t="inlineStr"/>
     </row>
     <row r="229">
       <c r="A229" s="5" t="n">
@@ -14107,7 +13940,6 @@
           <t>Heritage apparel brand recapitalized under a brand-management firm with an explicit growth mandate; fits profile of brands newly funded for expansion.</t>
         </is>
       </c>
-      <c r="P229" t="inlineStr"/>
     </row>
     <row r="230">
       <c r="A230" s="5" t="n">
@@ -14179,7 +14011,6 @@
           <t>One of 2026's largest D2C consumer raises, pushing valuation past $10B; classic profile of a scaled, well-funded consumer brand entering major sponsorship consideration.</t>
         </is>
       </c>
-      <c r="P230" t="inlineStr"/>
     </row>
     <row r="231">
       <c r="A231" s="4" t="inlineStr">
@@ -14250,7 +14081,6 @@
           <t>Background-check/identity-verification competitor to Checkr/HireRight already on the list; revenue ~$700M clears the core revenue gate.</t>
         </is>
       </c>
-      <c r="P232" t="inlineStr"/>
     </row>
     <row r="233">
       <c r="A233" s="5" t="n">
@@ -14314,7 +14144,6 @@
           <t>Major engineering/inspection firm for transport and venue infrastructure, motorsport-circuit adjacent; revenue &gt;$4B, core.</t>
         </is>
       </c>
-      <c r="P233" t="inlineStr"/>
     </row>
     <row r="234">
       <c r="A234" s="4" t="inlineStr">
@@ -14385,7 +14214,6 @@
           <t>Long-established food-industry weighing/packaging equipment maker with revenue above the $200M core threshold; APAC growth ambitions make F1's Japanese/Asian race calendar attractive exposure.</t>
         </is>
       </c>
-      <c r="P235" t="inlineStr"/>
     </row>
     <row r="236">
       <c r="A236" s="5" t="n">
@@ -14449,7 +14277,6 @@
           <t>Finnish forest-industry group (~EUR5B revenue) producing fibre-based packaging board as an alternative to plastics; sustainability credentials fit F1's renewable-materials sponsorship positioning well.</t>
         </is>
       </c>
-      <c r="P236" t="inlineStr"/>
     </row>
     <row r="237">
       <c r="A237" s="5" t="n">
@@ -14513,7 +14340,6 @@
           <t>Global packaging-film manufacturer (~EUR1.5B revenue, ~6,000 staff) with an active recyclable-materials push, offering a sustainability angle comparable to other packaging sponsors in the space.</t>
         </is>
       </c>
-      <c r="P237" t="inlineStr"/>
     </row>
     <row r="238">
       <c r="A238" s="5" t="n">
@@ -14577,7 +14403,6 @@
           <t>Fortune 50 agribusiness/ingredients giant (~$85B revenue) supplying flavors, starches and proteins to food manufacturers alongside peers like Kerry and Tate &amp; Lyle already tracked in this category.</t>
         </is>
       </c>
-      <c r="P238" t="inlineStr"/>
     </row>
     <row r="239">
       <c r="A239" s="5" t="n">
@@ -14641,7 +14466,6 @@
           <t>NYSE-listed global oilseed/grain processor (~$50B revenue) supplying edible oils and ingredients to the food industry; scale and international footprint suit a global sponsorship platform like F1.</t>
         </is>
       </c>
-      <c r="P239" t="inlineStr"/>
     </row>
     <row r="240">
       <c r="A240" s="5" t="n">
@@ -14705,7 +14529,6 @@
           <t>Asia's largest agribusiness group (~$60B revenue) spanning edible oils, food processing and packaging; strong APAC growth story aligns with F1's expanding Asian race calendar and fan base.</t>
         </is>
       </c>
-      <c r="P240" t="inlineStr"/>
     </row>
     <row r="241">
       <c r="A241" s="5" t="n">
@@ -14769,7 +14592,6 @@
           <t>Privately held but publicly reported ~$160B-revenue food and agriculture conglomerate; scale far exceeds the core gate, and its ingredient/packaging supply-chain footprint mirrors sponsors already tracked.</t>
         </is>
       </c>
-      <c r="P241" t="inlineStr"/>
     </row>
     <row r="242">
       <c r="A242" s="4" t="inlineStr">
@@ -14848,7 +14670,6 @@
           <t>Rapidly scaling European defense-AI drone maker with large capital base looking to raise its profile globally.</t>
         </is>
       </c>
-      <c r="P243" t="inlineStr"/>
     </row>
     <row r="244">
       <c r="A244" s="5" t="n">
@@ -14920,7 +14741,6 @@
           <t>Newly minted unicorn with a 'designed &amp; assembled in America' manufacturing story is building consumer and industrial-buyer awareness fast -- F1's engineering-performance narrative is an on-brand amplifier for a factory-automation challenger brand.</t>
         </is>
       </c>
-      <c r="P244" t="inlineStr"/>
     </row>
     <row r="245">
       <c r="A245" s="5" t="n">
@@ -14992,7 +14812,6 @@
           <t>One of the largest mobility capital events of the window; autonomous-driving technology leadership is a natural narrative fit for F1's technology-partner tier and does not conflict with existing F1 logistics/airline sponsors.</t>
         </is>
       </c>
-      <c r="P245" t="inlineStr"/>
     </row>
     <row r="246">
       <c r="A246" s="5" t="n">
@@ -15064,7 +14883,6 @@
           <t>Fresh $1.7B war chest; physical-AI narrative</t>
         </is>
       </c>
-      <c r="P246" t="inlineStr"/>
     </row>
     <row r="247">
       <c r="A247" s="5" t="n">
@@ -15136,7 +14954,6 @@
           <t>Fast-rising physical-AI robotics brand with ex-DeepMind/Boston Dynamics pedigree seeking global visibility.</t>
         </is>
       </c>
-      <c r="P247" t="inlineStr"/>
     </row>
     <row r="248">
       <c r="A248" s="5" t="n">
@@ -15208,7 +15025,6 @@
           <t>Newly-unicorn robotics/physical AI company with fresh capital seeking to build a recognizable global brand.</t>
         </is>
       </c>
-      <c r="P248" t="inlineStr"/>
     </row>
     <row r="249">
       <c r="A249" s="5" t="n">
@@ -15280,7 +15096,6 @@
           <t>Newly capitalized industrial-robotics AI startup working directly with an automaker (Rivian) on production-line data - directly relevant to F1 teams' own factory and manufacturing operations.</t>
         </is>
       </c>
-      <c r="P249" t="inlineStr"/>
     </row>
     <row r="250">
       <c r="A250" s="5" t="n">
@@ -15352,7 +15167,6 @@
           <t>A Swiss-engineered autonomy unicorn selling precision and safety to global construction and materials firms fits well with F1's engineering-precision brand halo, especially for a European team seeking industrial-tech sponsors.</t>
         </is>
       </c>
-      <c r="P250" t="inlineStr"/>
     </row>
     <row r="251">
       <c r="A251" s="5" t="n">
@@ -15424,7 +15238,144 @@
           <t>Newly minted construction-tech unicorn automating heavy equipment; engineering-precision and autonomy narrative aligns well with F1's performance-engineering brand positioning, unclaimed category (no current F1 construction/robotics sponsor).</t>
         </is>
       </c>
-      <c r="P251" t="inlineStr"/>
+    </row>
+    <row r="252">
+      <c r="A252" s="9" t="n">
+        <v>208</v>
+      </c>
+      <c r="B252" s="9" t="inlineStr">
+        <is>
+          <t>17 AI Cloud &amp; Data</t>
+        </is>
+      </c>
+      <c r="C252" s="9" t="inlineStr"/>
+      <c r="D252" s="9" t="n">
+        <v>52</v>
+      </c>
+      <c r="E252" s="9" t="inlineStr">
+        <is>
+          <t>Manual (you spotted it)</t>
+        </is>
+      </c>
+      <c r="F252" s="9" t="inlineStr">
+        <is>
+          <t>CuspAI</t>
+        </is>
+      </c>
+      <c r="G252" s="9" t="inlineStr">
+        <is>
+          <t>cusp.ai</t>
+        </is>
+      </c>
+      <c r="H252" s="9" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+      <c r="I252" s="9" t="inlineStr">
+        <is>
+          <t>AI materials discovery</t>
+        </is>
+      </c>
+      <c r="J252" s="10" t="inlineStr">
+        <is>
+          <t>$450M Series B at $2.6B (Kleiner/NEA/Bezos/AMD Ventures)</t>
+        </is>
+      </c>
+      <c r="K252" s="9" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="L252" s="9" t="inlineStr">
+        <is>
+          <t>$450M</t>
+        </is>
+      </c>
+      <c r="M252" s="9" t="inlineStr">
+        <is>
+          <t>~150</t>
+        </is>
+      </c>
+      <c r="N252" s="10" t="inlineStr">
+        <is>
+          <t>Deep-tech halo; UK home race; AMD compute tie-in</t>
+        </is>
+      </c>
+      <c r="O252" s="9" t="inlineStr">
+        <is>
+          <t>verified 20 Sep 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" s="9" t="n">
+        <v>209</v>
+      </c>
+      <c r="B253" s="9" t="inlineStr">
+        <is>
+          <t>AI Agents tab</t>
+        </is>
+      </c>
+      <c r="C253" s="9" t="inlineStr"/>
+      <c r="D253" s="9" t="n">
+        <v>60</v>
+      </c>
+      <c r="E253" s="9" t="inlineStr">
+        <is>
+          <t>Manual (you spotted it)</t>
+        </is>
+      </c>
+      <c r="F253" s="9" t="inlineStr">
+        <is>
+          <t>Wonderful</t>
+        </is>
+      </c>
+      <c r="G253" s="9" t="inlineStr">
+        <is>
+          <t>wonderful.ai</t>
+        </is>
+      </c>
+      <c r="H253" s="9" t="inlineStr">
+        <is>
+          <t>Israel / Netherlands</t>
+        </is>
+      </c>
+      <c r="I253" s="9" t="inlineStr">
+        <is>
+          <t>Enterprise AI OS / agent orchestration</t>
+        </is>
+      </c>
+      <c r="J253" s="10" t="inlineStr">
+        <is>
+          <t>$550M Series C at $5B (Insight-led; Salesforce minority investor - flag)</t>
+        </is>
+      </c>
+      <c r="K253" s="9" t="inlineStr">
+        <is>
+          <t>2 Sep 2026</t>
+        </is>
+      </c>
+      <c r="L253" s="9" t="inlineStr">
+        <is>
+          <t>$550M</t>
+        </is>
+      </c>
+      <c r="M253" s="9" t="inlineStr">
+        <is>
+          <t>~650</t>
+        </is>
+      </c>
+      <c r="N253" s="10" t="inlineStr">
+        <is>
+          <t>Agent-orchestration seat open on grid; 35+ markets</t>
+        </is>
+      </c>
+      <c r="O253" s="9" t="inlineStr">
+        <is>
+          <t>verified 20 Sep 2026</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="41">

</xml_diff>